<commit_message>
Day 32 — Capital Allocation Report
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -876,7 +876,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2532,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3893,7 +3893,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4468,7 +4468,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>

</xml_diff>